<commit_message>
refactor(#7) : 엑셀 셀 변경
출결, 봉사 등 필요없는 정보 삭제, 3학년 2학기 추가, 2차 전형 이름 변경
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/xlsx/1차전형결과.xlsx
+++ b/src/main/resources/templates/xlsx/1차전형결과.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jeon-yujin/Documents/workspace/backend/springboot/maru/src/main/resources/templates/xlsx/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hsm/Documents/백엔드/haeundae-marubase/src/main/resources/templates/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{851CB714-6559-5E4A-832A-5C8BB5C4FBD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B7B39D-785E-3E4B-903E-F3BE5BFA7363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15240" yWindow="740" windowWidth="15000" windowHeight="18900" xr2:uid="{7690012B-BFFA-3C48-824D-509550F219F4}"/>
+    <workbookView xWindow="13800" yWindow="500" windowWidth="15000" windowHeight="16540" xr2:uid="{7690012B-BFFA-3C48-824D-509550F219F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>수험번호</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -95,14 +95,6 @@
   </si>
   <si>
     <t>출결상황</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>봉사활동</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>가산점</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -566,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C8EB960-16E4-4546-BE22-CABF45F1D2EB}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="2" width="9.140625" bestFit="1" customWidth="1"/>
@@ -579,12 +571,11 @@
     <col min="10" max="10" width="16" customWidth="1"/>
     <col min="11" max="11" width="16.5703125" customWidth="1"/>
     <col min="12" max="12" width="9.5703125" customWidth="1"/>
-    <col min="13" max="15" width="9" customWidth="1"/>
-    <col min="16" max="16" width="7.42578125" customWidth="1"/>
-    <col min="17" max="17" width="9.42578125" customWidth="1"/>
+    <col min="13" max="14" width="9" customWidth="1"/>
+    <col min="15" max="15" width="9.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="30" customHeight="1">
+    <row r="1" spans="1:15" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
@@ -611,11 +602,9 @@
         <v>12</v>
       </c>
       <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="5"/>
+      <c r="O1" s="5"/>
     </row>
-    <row r="2" spans="1:17" ht="30" customHeight="1">
+    <row r="2" spans="1:15" ht="30" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
       <c r="C2" s="1" t="s">
@@ -632,7 +621,7 @@
         <v>8</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>10</v>
@@ -644,7 +633,7 @@
         <v>9</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>13</v>
@@ -654,22 +643,16 @@
       </c>
       <c r="O2" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="M1:O1"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:E2"/>
     <mergeCell ref="F1:L1"/>
-    <mergeCell ref="M1:Q1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor(#97) : 액셀 형식 변경
액셀 졸업 날짜 수청에 따라 컬럼 길이와 2차 전형 이후 면접 번호를 추가했습니다.
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/xlsx/1차전형결과.xlsx
+++ b/src/main/resources/templates/xlsx/1차전형결과.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hsm/Documents/백엔드/haeundae-marubase/src/main/resources/templates/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2B7B39D-785E-3E4B-903E-F3BE5BFA7363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48EC1F50-2B66-8E4E-AF4F-0AD84547B52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13800" yWindow="500" windowWidth="15000" windowHeight="16540" xr2:uid="{7690012B-BFFA-3C48-824D-509550F219F4}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16500" xr2:uid="{7690012B-BFFA-3C48-824D-509550F219F4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -218,9 +218,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -228,6 +225,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -568,7 +568,7 @@
     <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.7109375" customWidth="1"/>
     <col min="9" max="9" width="21.85546875" customWidth="1"/>
-    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="10" max="10" width="24.85546875" customWidth="1"/>
     <col min="11" max="11" width="16.5703125" customWidth="1"/>
     <col min="12" max="12" width="9.5703125" customWidth="1"/>
     <col min="13" max="14" width="9" customWidth="1"/>
@@ -576,44 +576,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2" t="s">
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4"/>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="4"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="3" t="s">
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="4"/>
-      <c r="O1" s="5"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" ht="30" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
       <c r="C2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="2"/>
+      <c r="E2" s="5"/>
       <c r="F2" s="1" t="s">
         <v>1</v>
       </c>

</xml_diff>